<commit_message>
fix: corrigir renomeacao de colunas trocadas em gerar_relatorio_indicadores
pivot_table ordena as colunas alfabeticamente (CDI, IGP-M, IPCA, Selic),
mas o codigo renomeava por posicao assumindo a ordem (CDI, IPCA, IGP-M,
Selic). Resultado: os valores de IPCA e IGP-M saiam trocados no Excel
exportado (Selic nao era afetada, ja que ficava na ultima posicao nos
dois casos). Troquei para renomear por nome do indicador (rename por
dict), robusto independente da ordem que o pivot_table devolver.

Reexportei relatorio_indicadores.xlsx com a correcao aplicada.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/relatorio_indicadores.xlsx
+++ b/relatorio_indicadores.xlsx
@@ -429,12 +429,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>IGP-M (% mês)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>IPCA (% mês)</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>IGP-M (% mês)</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">

</xml_diff>

<commit_message>
feat: integrar modulo de Opcoes B3 e ajustes de carteira/investidas
Adiciona modules/opcoes (Black-Scholes, IV/HV, screener, backtest) integrado como aba no app.py. Ajustes em carteira.py e investidas.py, e regeneracao dos relatorios Excel.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/relatorio_indicadores.xlsx
+++ b/relatorio_indicadores.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -752,11 +752,7 @@
           <t>01/07/2026</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>0.05%</t>
-        </is>
-      </c>
+      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>-1.16%</t>
@@ -772,7 +768,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>02/07/2026</t>
+          <t>01/07/2026</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -787,7 +783,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>03/07/2026</t>
+          <t>02/07/2026</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -802,7 +798,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>06/07/2026</t>
+          <t>03/07/2026</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -817,7 +813,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>07/07/2026</t>
+          <t>06/07/2026</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -832,7 +828,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>08/07/2026</t>
+          <t>07/07/2026</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -847,7 +843,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>09/07/2026</t>
+          <t>08/07/2026</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -862,7 +858,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>10/07/2026</t>
+          <t>09/07/2026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -877,82 +873,82 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>25/07/2026</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr"/>
+          <t>10/07/2026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>0.05%</t>
+        </is>
+      </c>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>14.25%</t>
-        </is>
-      </c>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>26/07/2026</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr"/>
+          <t>13/07/2026</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>0.05%</t>
+        </is>
+      </c>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>14.25%</t>
-        </is>
-      </c>
+      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>27/07/2026</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr"/>
+          <t>22/07/2026</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>0.05%</t>
+        </is>
+      </c>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>14.25%</t>
-        </is>
-      </c>
+      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr"/>
+          <t>23/07/2026</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>0.05%</t>
+        </is>
+      </c>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>14.25%</t>
-        </is>
-      </c>
+      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr"/>
+          <t>24/07/2026</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>0.05%</t>
+        </is>
+      </c>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>14.25%</t>
-        </is>
-      </c>
+      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>30/07/2026</t>
+          <t>25/07/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
@@ -967,7 +963,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>31/07/2026</t>
+          <t>26/07/2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -982,26 +978,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>01/08/2026</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr"/>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>-0.22%</t>
-        </is>
-      </c>
+          <t>27/07/2026</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>0.05%</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>14.25%</t>
-        </is>
-      </c>
+      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>02/08/2026</t>
+          <t>27/07/2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
@@ -1016,22 +1008,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>03/08/2026</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr"/>
+          <t>28/07/2026</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>0.05%</t>
+        </is>
+      </c>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>14.25%</t>
-        </is>
-      </c>
+      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>04/08/2026</t>
+          <t>28/07/2026</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
@@ -1046,37 +1038,37 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr"/>
+          <t>29/07/2026</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>0.05%</t>
+        </is>
+      </c>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>14.25%</t>
-        </is>
-      </c>
+      <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>12/08/2026</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>0.05%</t>
-        </is>
-      </c>
+          <t>29/07/2026</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>14.25%</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>13/08/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1091,22 +1083,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>14/08/2026</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>0.05%</t>
-        </is>
-      </c>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>14.25%</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>17/08/2026</t>
+          <t>31/07/2026</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1121,67 +1113,67 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>18/08/2026</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>0.05%</t>
-        </is>
-      </c>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>14.25%</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>19/08/2026</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>0.05%</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr"/>
+          <t>01/08/2026</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>-0.22%</t>
+        </is>
+      </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>20/08/2026</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>0.05%</t>
-        </is>
-      </c>
+          <t>01/08/2026</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>14.25%</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>21/08/2026</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>0.05%</t>
-        </is>
-      </c>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>14.25%</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>24/08/2026</t>
+          <t>03/08/2026</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1196,22 +1188,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>25/08/2026</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>0.05%</t>
-        </is>
-      </c>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>14.25%</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>04/08/2026</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1226,37 +1218,37 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>27/08/2026</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>0.05%</t>
-        </is>
-      </c>
+          <t>04/08/2026</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>14.25%</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr"/>
+          <t>05/08/2026</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>0.05%</t>
+        </is>
+      </c>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>14.00%</t>
-        </is>
-      </c>
+      <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>06/09/2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
       <c r="B52" t="inlineStr"/>
@@ -1264,155 +1256,380 @@
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
-          <t>14.00%</t>
+          <t>14.25%</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr"/>
+          <t>06/08/2026</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>0.05%</t>
+        </is>
+      </c>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>14.00%</t>
-        </is>
-      </c>
+      <c r="E53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr"/>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>0.05%</t>
+        </is>
+      </c>
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>14.00%</t>
-        </is>
-      </c>
+      <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr"/>
+          <t>13/08/2026</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>0.05%</t>
+        </is>
+      </c>
       <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>14.00%</t>
-        </is>
-      </c>
+      <c r="E55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr"/>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>0.05%</t>
+        </is>
+      </c>
       <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>14.00%</t>
-        </is>
-      </c>
+      <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr"/>
+          <t>17/08/2026</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>0.05%</t>
+        </is>
+      </c>
       <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>14.00%</t>
-        </is>
-      </c>
+      <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>12/09/2026</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr"/>
+          <t>18/08/2026</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>0.05%</t>
+        </is>
+      </c>
       <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>14.00%</t>
-        </is>
-      </c>
+      <c r="E58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr"/>
+          <t>19/08/2026</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>0.05%</t>
+        </is>
+      </c>
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr"/>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>14.00%</t>
-        </is>
-      </c>
+      <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr"/>
+          <t>20/08/2026</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>0.05%</t>
+        </is>
+      </c>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>14.00%</t>
-        </is>
-      </c>
+      <c r="E60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr"/>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>0.05%</t>
+        </is>
+      </c>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>14.00%</t>
-        </is>
-      </c>
+      <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>16/09/2026</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr"/>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>0.05%</t>
+        </is>
+      </c>
       <c r="C62" t="inlineStr"/>
       <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr">
+      <c r="E62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>0.05%</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>26/08/2026</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>0.05%</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>0.05%</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>05/09/2026</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr"/>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>14.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>06/09/2026</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>14.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>07/09/2026</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr"/>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>14.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>14.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>14.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr"/>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>14.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>14.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>12/09/2026</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr"/>
+      <c r="C73" t="inlineStr"/>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>14.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr"/>
+      <c r="C74" t="inlineStr"/>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>14.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr"/>
+      <c r="C75" t="inlineStr"/>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>14.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>15/09/2026</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr"/>
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>14.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr"/>
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr">
         <is>
           <t>14.00%</t>
         </is>

</xml_diff>